<commit_message>
Added admin & user auth
</commit_message>
<xml_diff>
--- a/backend/data/excels/17-02-2026/DEPO_february.xlsx
+++ b/backend/data/excels/17-02-2026/DEPO_february.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Администратор\Desktop\IT_projects\uzonia\backend\data\input_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kakhramon/Desktop/CBU/uzonia/backend/data/excels/17-02-2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75FD6397-DF0D-4944-9C6A-56F7F85C288B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07F8E806-2355-0D48-B8C6-74EDC0AE5411}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-1425" windowWidth="38640" windowHeight="21120" xr2:uid="{D8556142-6755-46FB-802F-D3FBD9EE2E33}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15940" xr2:uid="{D8556142-6755-46FB-802F-D3FBD9EE2E33}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="11">
   <si>
     <t>Код сделки</t>
   </si>
@@ -69,6 +69,9 @@
   </si>
   <si>
     <t>UZS</t>
+  </si>
+  <si>
+    <t>bank</t>
   </si>
 </sst>
 </file>
@@ -78,7 +81,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd\.mm\.yyyy"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -106,6 +109,12 @@
       <name val="Tahoma"/>
       <family val="2"/>
       <charset val="204"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -173,9 +182,6 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="39" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -190,9 +196,10 @@
     <xf numFmtId="39" fontId="1" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Обычный 2" xfId="1" xr:uid="{01B81631-4321-4BE9-888C-3F9DAED13761}"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -209,9 +216,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Стандартная">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -249,7 +256,7 @@
         <a:srgbClr val="96607D"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Стандартная">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
         <a:ea typeface=""/>
@@ -355,7 +362,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Стандартная">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -526,19 +533,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43ECFB80-075C-4577-B2A1-07FCC1D20F4B}">
   <dimension ref="A1:I5"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.85546875" customWidth="1"/>
-    <col min="2" max="2" width="16.85546875" customWidth="1"/>
-    <col min="3" max="3" width="9.42578125" customWidth="1"/>
-    <col min="5" max="5" width="13.42578125" customWidth="1"/>
-    <col min="6" max="6" width="22.28515625" customWidth="1"/>
-    <col min="7" max="7" width="11.7109375" customWidth="1"/>
-    <col min="8" max="8" width="18.140625" customWidth="1"/>
-    <col min="9" max="9" width="14.7109375" customWidth="1"/>
+    <col min="1" max="1" width="13.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="9.5" customWidth="1"/>
+    <col min="5" max="5" width="13.5" customWidth="1"/>
+    <col min="6" max="6" width="22.33203125" customWidth="1"/>
+    <col min="7" max="7" width="11.6640625" customWidth="1"/>
+    <col min="8" max="8" width="18.1640625" customWidth="1"/>
+    <col min="9" max="9" width="14.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="33.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="26" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -567,22 +574,26 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" s="9" customFormat="1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" s="8" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="3">
         <v>14818</v>
       </c>
       <c r="B2" s="4">
         <v>46070</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="6" t="s">
+      <c r="C2" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="7">
+      <c r="F2" s="6">
         <v>70000000000</v>
       </c>
-      <c r="G2" s="8">
+      <c r="G2" s="7">
         <v>13.5</v>
       </c>
       <c r="H2" s="4">
@@ -592,22 +603,26 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:9" s="9" customFormat="1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" s="8" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="3">
         <v>14819</v>
       </c>
       <c r="B3" s="4">
         <v>46070</v>
       </c>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="6" t="s">
+      <c r="C3" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="7">
+      <c r="F3" s="6">
         <v>149000000000</v>
       </c>
-      <c r="G3" s="8">
+      <c r="G3" s="7">
         <v>13.5</v>
       </c>
       <c r="H3" s="4">
@@ -617,22 +632,26 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:9" s="9" customFormat="1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" s="8" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="3">
         <v>14820</v>
       </c>
       <c r="B4" s="4">
         <v>46070</v>
       </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="6" t="s">
+      <c r="C4" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F4" s="10">
+      <c r="F4" s="9">
         <v>30000000000</v>
       </c>
-      <c r="G4" s="8">
+      <c r="G4" s="7">
         <v>13.5</v>
       </c>
       <c r="H4" s="4">
@@ -642,22 +661,26 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:9" s="9" customFormat="1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" s="8" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="3">
         <v>14821</v>
       </c>
       <c r="B5" s="4">
         <v>46070</v>
       </c>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="6" t="s">
+      <c r="C5" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="7">
+      <c r="F5" s="6">
         <v>3000000000</v>
       </c>
-      <c r="G5" s="8">
+      <c r="G5" s="7">
         <v>14</v>
       </c>
       <c r="H5" s="4">

</xml_diff>